<commit_message>
Two templates, tab-per-day dates, and three new tests
- Two template downloads: "one tab" (Date column) and "tab per day"
  (one tab per testing day, named with the date, e.g. 1.24.26)
- Reads the testing date from the tab name when a tab has no Date column
- New tests: Safety Bar Squat (estimated max), Push-Up and Chin-Up (reps)
- Templates include the new columns and a gray example row (skipped on upload)
- No-data message explains both layouts

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/testing-template.xlsx
+++ b/testing-template.xlsx
@@ -20,7 +20,7 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="m/d/yy"/>
   </numFmts>
-  <fonts count="3">
+  <fonts count="4">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
@@ -33,10 +33,14 @@
       <color rgb="00FFFFFF"/>
     </font>
     <font>
+      <i val="1"/>
+      <color rgb="007A8494"/>
+    </font>
+    <font>
       <b val="1"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill/>
     </fill>
@@ -45,7 +49,12 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="000B2A4A"/>
+        <fgColor rgb="00003764"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00EEF3F8"/>
       </patternFill>
     </fill>
   </fills>
@@ -61,13 +70,16 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="4">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="49" fontId="2" fillId="3" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="3" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
@@ -433,7 +445,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:K500"/>
+  <dimension ref="A1:N500"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="11" customWidth="1" min="1" max="1"/>
@@ -447,6 +459,9 @@
     <col width="12" customWidth="1" min="9" max="9"/>
     <col width="12" customWidth="1" min="10" max="10"/>
     <col width="10" customWidth="1" min="11" max="11"/>
+    <col width="16" customWidth="1" min="12" max="12"/>
+    <col width="10" customWidth="1" min="13" max="13"/>
+    <col width="10" customWidth="1" min="14" max="14"/>
   </cols>
   <sheetData>
     <row r="1">
@@ -505,1503 +520,1583 @@
           <t>Bench</t>
         </is>
       </c>
+      <c r="L1" s="1" t="inlineStr">
+        <is>
+          <t>Safety Bar Squat</t>
+        </is>
+      </c>
+      <c r="M1" s="1" t="inlineStr">
+        <is>
+          <t>Push-Up</t>
+        </is>
+      </c>
+      <c r="N1" s="1" t="inlineStr">
+        <is>
+          <t>Chin-Up</t>
+        </is>
+      </c>
     </row>
     <row r="2">
-      <c r="A2" s="2" t="n"/>
+      <c r="A2" s="2" t="inlineStr">
+        <is>
+          <t>1/24/26</t>
+        </is>
+      </c>
+      <c r="B2" s="2" t="n"/>
+      <c r="C2" s="2" t="inlineStr">
+        <is>
+          <t>Football</t>
+        </is>
+      </c>
+      <c r="D2" s="2" t="inlineStr">
+        <is>
+          <t>WR</t>
+        </is>
+      </c>
+      <c r="E2" s="2" t="inlineStr">
+        <is>
+          <t>1.62</t>
+        </is>
+      </c>
+      <c r="F2" s="2" t="inlineStr">
+        <is>
+          <t>28.4</t>
+        </is>
+      </c>
+      <c r="G2" s="2" t="inlineStr">
+        <is>
+          <t>8'11</t>
+        </is>
+      </c>
+      <c r="H2" s="2" t="inlineStr">
+        <is>
+          <t>315x5</t>
+        </is>
+      </c>
+      <c r="I2" s="2" t="inlineStr">
+        <is>
+          <t>275x4</t>
+        </is>
+      </c>
+      <c r="J2" s="2" t="inlineStr">
+        <is>
+          <t>405x3</t>
+        </is>
+      </c>
+      <c r="K2" s="2" t="inlineStr">
+        <is>
+          <t>225x5</t>
+        </is>
+      </c>
+      <c r="L2" s="2" t="inlineStr">
+        <is>
+          <t>335x5</t>
+        </is>
+      </c>
+      <c r="M2" s="2" t="inlineStr">
+        <is>
+          <t>31</t>
+        </is>
+      </c>
+      <c r="N2" s="2" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
     </row>
     <row r="3">
-      <c r="A3" s="2" t="n"/>
+      <c r="A3" s="3" t="n"/>
     </row>
     <row r="4">
-      <c r="A4" s="2" t="n"/>
+      <c r="A4" s="3" t="n"/>
     </row>
     <row r="5">
-      <c r="A5" s="2" t="n"/>
+      <c r="A5" s="3" t="n"/>
     </row>
     <row r="6">
-      <c r="A6" s="2" t="n"/>
+      <c r="A6" s="3" t="n"/>
     </row>
     <row r="7">
-      <c r="A7" s="2" t="n"/>
+      <c r="A7" s="3" t="n"/>
     </row>
     <row r="8">
-      <c r="A8" s="2" t="n"/>
+      <c r="A8" s="3" t="n"/>
     </row>
     <row r="9">
-      <c r="A9" s="2" t="n"/>
+      <c r="A9" s="3" t="n"/>
     </row>
     <row r="10">
-      <c r="A10" s="2" t="n"/>
+      <c r="A10" s="3" t="n"/>
     </row>
     <row r="11">
-      <c r="A11" s="2" t="n"/>
+      <c r="A11" s="3" t="n"/>
     </row>
     <row r="12">
-      <c r="A12" s="2" t="n"/>
+      <c r="A12" s="3" t="n"/>
     </row>
     <row r="13">
-      <c r="A13" s="2" t="n"/>
+      <c r="A13" s="3" t="n"/>
     </row>
     <row r="14">
-      <c r="A14" s="2" t="n"/>
+      <c r="A14" s="3" t="n"/>
     </row>
     <row r="15">
-      <c r="A15" s="2" t="n"/>
+      <c r="A15" s="3" t="n"/>
     </row>
     <row r="16">
-      <c r="A16" s="2" t="n"/>
+      <c r="A16" s="3" t="n"/>
     </row>
     <row r="17">
-      <c r="A17" s="2" t="n"/>
+      <c r="A17" s="3" t="n"/>
     </row>
     <row r="18">
-      <c r="A18" s="2" t="n"/>
+      <c r="A18" s="3" t="n"/>
     </row>
     <row r="19">
-      <c r="A19" s="2" t="n"/>
+      <c r="A19" s="3" t="n"/>
     </row>
     <row r="20">
-      <c r="A20" s="2" t="n"/>
+      <c r="A20" s="3" t="n"/>
     </row>
     <row r="21">
-      <c r="A21" s="2" t="n"/>
+      <c r="A21" s="3" t="n"/>
     </row>
     <row r="22">
-      <c r="A22" s="2" t="n"/>
+      <c r="A22" s="3" t="n"/>
     </row>
     <row r="23">
-      <c r="A23" s="2" t="n"/>
+      <c r="A23" s="3" t="n"/>
     </row>
     <row r="24">
-      <c r="A24" s="2" t="n"/>
+      <c r="A24" s="3" t="n"/>
     </row>
     <row r="25">
-      <c r="A25" s="2" t="n"/>
+      <c r="A25" s="3" t="n"/>
     </row>
     <row r="26">
-      <c r="A26" s="2" t="n"/>
+      <c r="A26" s="3" t="n"/>
     </row>
     <row r="27">
-      <c r="A27" s="2" t="n"/>
+      <c r="A27" s="3" t="n"/>
     </row>
     <row r="28">
-      <c r="A28" s="2" t="n"/>
+      <c r="A28" s="3" t="n"/>
     </row>
     <row r="29">
-      <c r="A29" s="2" t="n"/>
+      <c r="A29" s="3" t="n"/>
     </row>
     <row r="30">
-      <c r="A30" s="2" t="n"/>
+      <c r="A30" s="3" t="n"/>
     </row>
     <row r="31">
-      <c r="A31" s="2" t="n"/>
+      <c r="A31" s="3" t="n"/>
     </row>
     <row r="32">
-      <c r="A32" s="2" t="n"/>
+      <c r="A32" s="3" t="n"/>
     </row>
     <row r="33">
-      <c r="A33" s="2" t="n"/>
+      <c r="A33" s="3" t="n"/>
     </row>
     <row r="34">
-      <c r="A34" s="2" t="n"/>
+      <c r="A34" s="3" t="n"/>
     </row>
     <row r="35">
-      <c r="A35" s="2" t="n"/>
+      <c r="A35" s="3" t="n"/>
     </row>
     <row r="36">
-      <c r="A36" s="2" t="n"/>
+      <c r="A36" s="3" t="n"/>
     </row>
     <row r="37">
-      <c r="A37" s="2" t="n"/>
+      <c r="A37" s="3" t="n"/>
     </row>
     <row r="38">
-      <c r="A38" s="2" t="n"/>
+      <c r="A38" s="3" t="n"/>
     </row>
     <row r="39">
-      <c r="A39" s="2" t="n"/>
+      <c r="A39" s="3" t="n"/>
     </row>
     <row r="40">
-      <c r="A40" s="2" t="n"/>
+      <c r="A40" s="3" t="n"/>
     </row>
     <row r="41">
-      <c r="A41" s="2" t="n"/>
+      <c r="A41" s="3" t="n"/>
     </row>
     <row r="42">
-      <c r="A42" s="2" t="n"/>
+      <c r="A42" s="3" t="n"/>
     </row>
     <row r="43">
-      <c r="A43" s="2" t="n"/>
+      <c r="A43" s="3" t="n"/>
     </row>
     <row r="44">
-      <c r="A44" s="2" t="n"/>
+      <c r="A44" s="3" t="n"/>
     </row>
     <row r="45">
-      <c r="A45" s="2" t="n"/>
+      <c r="A45" s="3" t="n"/>
     </row>
     <row r="46">
-      <c r="A46" s="2" t="n"/>
+      <c r="A46" s="3" t="n"/>
     </row>
     <row r="47">
-      <c r="A47" s="2" t="n"/>
+      <c r="A47" s="3" t="n"/>
     </row>
     <row r="48">
-      <c r="A48" s="2" t="n"/>
+      <c r="A48" s="3" t="n"/>
     </row>
     <row r="49">
-      <c r="A49" s="2" t="n"/>
+      <c r="A49" s="3" t="n"/>
     </row>
     <row r="50">
-      <c r="A50" s="2" t="n"/>
+      <c r="A50" s="3" t="n"/>
     </row>
     <row r="51">
-      <c r="A51" s="2" t="n"/>
+      <c r="A51" s="3" t="n"/>
     </row>
     <row r="52">
-      <c r="A52" s="2" t="n"/>
+      <c r="A52" s="3" t="n"/>
     </row>
     <row r="53">
-      <c r="A53" s="2" t="n"/>
+      <c r="A53" s="3" t="n"/>
     </row>
     <row r="54">
-      <c r="A54" s="2" t="n"/>
+      <c r="A54" s="3" t="n"/>
     </row>
     <row r="55">
-      <c r="A55" s="2" t="n"/>
+      <c r="A55" s="3" t="n"/>
     </row>
     <row r="56">
-      <c r="A56" s="2" t="n"/>
+      <c r="A56" s="3" t="n"/>
     </row>
     <row r="57">
-      <c r="A57" s="2" t="n"/>
+      <c r="A57" s="3" t="n"/>
     </row>
     <row r="58">
-      <c r="A58" s="2" t="n"/>
+      <c r="A58" s="3" t="n"/>
     </row>
     <row r="59">
-      <c r="A59" s="2" t="n"/>
+      <c r="A59" s="3" t="n"/>
     </row>
     <row r="60">
-      <c r="A60" s="2" t="n"/>
+      <c r="A60" s="3" t="n"/>
     </row>
     <row r="61">
-      <c r="A61" s="2" t="n"/>
+      <c r="A61" s="3" t="n"/>
     </row>
     <row r="62">
-      <c r="A62" s="2" t="n"/>
+      <c r="A62" s="3" t="n"/>
     </row>
     <row r="63">
-      <c r="A63" s="2" t="n"/>
+      <c r="A63" s="3" t="n"/>
     </row>
     <row r="64">
-      <c r="A64" s="2" t="n"/>
+      <c r="A64" s="3" t="n"/>
     </row>
     <row r="65">
-      <c r="A65" s="2" t="n"/>
+      <c r="A65" s="3" t="n"/>
     </row>
     <row r="66">
-      <c r="A66" s="2" t="n"/>
+      <c r="A66" s="3" t="n"/>
     </row>
     <row r="67">
-      <c r="A67" s="2" t="n"/>
+      <c r="A67" s="3" t="n"/>
     </row>
     <row r="68">
-      <c r="A68" s="2" t="n"/>
+      <c r="A68" s="3" t="n"/>
     </row>
     <row r="69">
-      <c r="A69" s="2" t="n"/>
+      <c r="A69" s="3" t="n"/>
     </row>
     <row r="70">
-      <c r="A70" s="2" t="n"/>
+      <c r="A70" s="3" t="n"/>
     </row>
     <row r="71">
-      <c r="A71" s="2" t="n"/>
+      <c r="A71" s="3" t="n"/>
     </row>
     <row r="72">
-      <c r="A72" s="2" t="n"/>
+      <c r="A72" s="3" t="n"/>
     </row>
     <row r="73">
-      <c r="A73" s="2" t="n"/>
+      <c r="A73" s="3" t="n"/>
     </row>
     <row r="74">
-      <c r="A74" s="2" t="n"/>
+      <c r="A74" s="3" t="n"/>
     </row>
     <row r="75">
-      <c r="A75" s="2" t="n"/>
+      <c r="A75" s="3" t="n"/>
     </row>
     <row r="76">
-      <c r="A76" s="2" t="n"/>
+      <c r="A76" s="3" t="n"/>
     </row>
     <row r="77">
-      <c r="A77" s="2" t="n"/>
+      <c r="A77" s="3" t="n"/>
     </row>
     <row r="78">
-      <c r="A78" s="2" t="n"/>
+      <c r="A78" s="3" t="n"/>
     </row>
     <row r="79">
-      <c r="A79" s="2" t="n"/>
+      <c r="A79" s="3" t="n"/>
     </row>
     <row r="80">
-      <c r="A80" s="2" t="n"/>
+      <c r="A80" s="3" t="n"/>
     </row>
     <row r="81">
-      <c r="A81" s="2" t="n"/>
+      <c r="A81" s="3" t="n"/>
     </row>
     <row r="82">
-      <c r="A82" s="2" t="n"/>
+      <c r="A82" s="3" t="n"/>
     </row>
     <row r="83">
-      <c r="A83" s="2" t="n"/>
+      <c r="A83" s="3" t="n"/>
     </row>
     <row r="84">
-      <c r="A84" s="2" t="n"/>
+      <c r="A84" s="3" t="n"/>
     </row>
     <row r="85">
-      <c r="A85" s="2" t="n"/>
+      <c r="A85" s="3" t="n"/>
     </row>
     <row r="86">
-      <c r="A86" s="2" t="n"/>
+      <c r="A86" s="3" t="n"/>
     </row>
     <row r="87">
-      <c r="A87" s="2" t="n"/>
+      <c r="A87" s="3" t="n"/>
     </row>
     <row r="88">
-      <c r="A88" s="2" t="n"/>
+      <c r="A88" s="3" t="n"/>
     </row>
     <row r="89">
-      <c r="A89" s="2" t="n"/>
+      <c r="A89" s="3" t="n"/>
     </row>
     <row r="90">
-      <c r="A90" s="2" t="n"/>
+      <c r="A90" s="3" t="n"/>
     </row>
     <row r="91">
-      <c r="A91" s="2" t="n"/>
+      <c r="A91" s="3" t="n"/>
     </row>
     <row r="92">
-      <c r="A92" s="2" t="n"/>
+      <c r="A92" s="3" t="n"/>
     </row>
     <row r="93">
-      <c r="A93" s="2" t="n"/>
+      <c r="A93" s="3" t="n"/>
     </row>
     <row r="94">
-      <c r="A94" s="2" t="n"/>
+      <c r="A94" s="3" t="n"/>
     </row>
     <row r="95">
-      <c r="A95" s="2" t="n"/>
+      <c r="A95" s="3" t="n"/>
     </row>
     <row r="96">
-      <c r="A96" s="2" t="n"/>
+      <c r="A96" s="3" t="n"/>
     </row>
     <row r="97">
-      <c r="A97" s="2" t="n"/>
+      <c r="A97" s="3" t="n"/>
     </row>
     <row r="98">
-      <c r="A98" s="2" t="n"/>
+      <c r="A98" s="3" t="n"/>
     </row>
     <row r="99">
-      <c r="A99" s="2" t="n"/>
+      <c r="A99" s="3" t="n"/>
     </row>
     <row r="100">
-      <c r="A100" s="2" t="n"/>
+      <c r="A100" s="3" t="n"/>
     </row>
     <row r="101">
-      <c r="A101" s="2" t="n"/>
+      <c r="A101" s="3" t="n"/>
     </row>
     <row r="102">
-      <c r="A102" s="2" t="n"/>
+      <c r="A102" s="3" t="n"/>
     </row>
     <row r="103">
-      <c r="A103" s="2" t="n"/>
+      <c r="A103" s="3" t="n"/>
     </row>
     <row r="104">
-      <c r="A104" s="2" t="n"/>
+      <c r="A104" s="3" t="n"/>
     </row>
     <row r="105">
-      <c r="A105" s="2" t="n"/>
+      <c r="A105" s="3" t="n"/>
     </row>
     <row r="106">
-      <c r="A106" s="2" t="n"/>
+      <c r="A106" s="3" t="n"/>
     </row>
     <row r="107">
-      <c r="A107" s="2" t="n"/>
+      <c r="A107" s="3" t="n"/>
     </row>
     <row r="108">
-      <c r="A108" s="2" t="n"/>
+      <c r="A108" s="3" t="n"/>
     </row>
     <row r="109">
-      <c r="A109" s="2" t="n"/>
+      <c r="A109" s="3" t="n"/>
     </row>
     <row r="110">
-      <c r="A110" s="2" t="n"/>
+      <c r="A110" s="3" t="n"/>
     </row>
     <row r="111">
-      <c r="A111" s="2" t="n"/>
+      <c r="A111" s="3" t="n"/>
     </row>
     <row r="112">
-      <c r="A112" s="2" t="n"/>
+      <c r="A112" s="3" t="n"/>
     </row>
     <row r="113">
-      <c r="A113" s="2" t="n"/>
+      <c r="A113" s="3" t="n"/>
     </row>
     <row r="114">
-      <c r="A114" s="2" t="n"/>
+      <c r="A114" s="3" t="n"/>
     </row>
     <row r="115">
-      <c r="A115" s="2" t="n"/>
+      <c r="A115" s="3" t="n"/>
     </row>
     <row r="116">
-      <c r="A116" s="2" t="n"/>
+      <c r="A116" s="3" t="n"/>
     </row>
     <row r="117">
-      <c r="A117" s="2" t="n"/>
+      <c r="A117" s="3" t="n"/>
     </row>
     <row r="118">
-      <c r="A118" s="2" t="n"/>
+      <c r="A118" s="3" t="n"/>
     </row>
     <row r="119">
-      <c r="A119" s="2" t="n"/>
+      <c r="A119" s="3" t="n"/>
     </row>
     <row r="120">
-      <c r="A120" s="2" t="n"/>
+      <c r="A120" s="3" t="n"/>
     </row>
     <row r="121">
-      <c r="A121" s="2" t="n"/>
+      <c r="A121" s="3" t="n"/>
     </row>
     <row r="122">
-      <c r="A122" s="2" t="n"/>
+      <c r="A122" s="3" t="n"/>
     </row>
     <row r="123">
-      <c r="A123" s="2" t="n"/>
+      <c r="A123" s="3" t="n"/>
     </row>
     <row r="124">
-      <c r="A124" s="2" t="n"/>
+      <c r="A124" s="3" t="n"/>
     </row>
     <row r="125">
-      <c r="A125" s="2" t="n"/>
+      <c r="A125" s="3" t="n"/>
     </row>
     <row r="126">
-      <c r="A126" s="2" t="n"/>
+      <c r="A126" s="3" t="n"/>
     </row>
     <row r="127">
-      <c r="A127" s="2" t="n"/>
+      <c r="A127" s="3" t="n"/>
     </row>
     <row r="128">
-      <c r="A128" s="2" t="n"/>
+      <c r="A128" s="3" t="n"/>
     </row>
     <row r="129">
-      <c r="A129" s="2" t="n"/>
+      <c r="A129" s="3" t="n"/>
     </row>
     <row r="130">
-      <c r="A130" s="2" t="n"/>
+      <c r="A130" s="3" t="n"/>
     </row>
     <row r="131">
-      <c r="A131" s="2" t="n"/>
+      <c r="A131" s="3" t="n"/>
     </row>
     <row r="132">
-      <c r="A132" s="2" t="n"/>
+      <c r="A132" s="3" t="n"/>
     </row>
     <row r="133">
-      <c r="A133" s="2" t="n"/>
+      <c r="A133" s="3" t="n"/>
     </row>
     <row r="134">
-      <c r="A134" s="2" t="n"/>
+      <c r="A134" s="3" t="n"/>
     </row>
     <row r="135">
-      <c r="A135" s="2" t="n"/>
+      <c r="A135" s="3" t="n"/>
     </row>
     <row r="136">
-      <c r="A136" s="2" t="n"/>
+      <c r="A136" s="3" t="n"/>
     </row>
     <row r="137">
-      <c r="A137" s="2" t="n"/>
+      <c r="A137" s="3" t="n"/>
     </row>
     <row r="138">
-      <c r="A138" s="2" t="n"/>
+      <c r="A138" s="3" t="n"/>
     </row>
     <row r="139">
-      <c r="A139" s="2" t="n"/>
+      <c r="A139" s="3" t="n"/>
     </row>
     <row r="140">
-      <c r="A140" s="2" t="n"/>
+      <c r="A140" s="3" t="n"/>
     </row>
     <row r="141">
-      <c r="A141" s="2" t="n"/>
+      <c r="A141" s="3" t="n"/>
     </row>
     <row r="142">
-      <c r="A142" s="2" t="n"/>
+      <c r="A142" s="3" t="n"/>
     </row>
     <row r="143">
-      <c r="A143" s="2" t="n"/>
+      <c r="A143" s="3" t="n"/>
     </row>
     <row r="144">
-      <c r="A144" s="2" t="n"/>
+      <c r="A144" s="3" t="n"/>
     </row>
     <row r="145">
-      <c r="A145" s="2" t="n"/>
+      <c r="A145" s="3" t="n"/>
     </row>
     <row r="146">
-      <c r="A146" s="2" t="n"/>
+      <c r="A146" s="3" t="n"/>
     </row>
     <row r="147">
-      <c r="A147" s="2" t="n"/>
+      <c r="A147" s="3" t="n"/>
     </row>
     <row r="148">
-      <c r="A148" s="2" t="n"/>
+      <c r="A148" s="3" t="n"/>
     </row>
     <row r="149">
-      <c r="A149" s="2" t="n"/>
+      <c r="A149" s="3" t="n"/>
     </row>
     <row r="150">
-      <c r="A150" s="2" t="n"/>
+      <c r="A150" s="3" t="n"/>
     </row>
     <row r="151">
-      <c r="A151" s="2" t="n"/>
+      <c r="A151" s="3" t="n"/>
     </row>
     <row r="152">
-      <c r="A152" s="2" t="n"/>
+      <c r="A152" s="3" t="n"/>
     </row>
     <row r="153">
-      <c r="A153" s="2" t="n"/>
+      <c r="A153" s="3" t="n"/>
     </row>
     <row r="154">
-      <c r="A154" s="2" t="n"/>
+      <c r="A154" s="3" t="n"/>
     </row>
     <row r="155">
-      <c r="A155" s="2" t="n"/>
+      <c r="A155" s="3" t="n"/>
     </row>
     <row r="156">
-      <c r="A156" s="2" t="n"/>
+      <c r="A156" s="3" t="n"/>
     </row>
     <row r="157">
-      <c r="A157" s="2" t="n"/>
+      <c r="A157" s="3" t="n"/>
     </row>
     <row r="158">
-      <c r="A158" s="2" t="n"/>
+      <c r="A158" s="3" t="n"/>
     </row>
     <row r="159">
-      <c r="A159" s="2" t="n"/>
+      <c r="A159" s="3" t="n"/>
     </row>
     <row r="160">
-      <c r="A160" s="2" t="n"/>
+      <c r="A160" s="3" t="n"/>
     </row>
     <row r="161">
-      <c r="A161" s="2" t="n"/>
+      <c r="A161" s="3" t="n"/>
     </row>
     <row r="162">
-      <c r="A162" s="2" t="n"/>
+      <c r="A162" s="3" t="n"/>
     </row>
     <row r="163">
-      <c r="A163" s="2" t="n"/>
+      <c r="A163" s="3" t="n"/>
     </row>
     <row r="164">
-      <c r="A164" s="2" t="n"/>
+      <c r="A164" s="3" t="n"/>
     </row>
     <row r="165">
-      <c r="A165" s="2" t="n"/>
+      <c r="A165" s="3" t="n"/>
     </row>
     <row r="166">
-      <c r="A166" s="2" t="n"/>
+      <c r="A166" s="3" t="n"/>
     </row>
     <row r="167">
-      <c r="A167" s="2" t="n"/>
+      <c r="A167" s="3" t="n"/>
     </row>
     <row r="168">
-      <c r="A168" s="2" t="n"/>
+      <c r="A168" s="3" t="n"/>
     </row>
     <row r="169">
-      <c r="A169" s="2" t="n"/>
+      <c r="A169" s="3" t="n"/>
     </row>
     <row r="170">
-      <c r="A170" s="2" t="n"/>
+      <c r="A170" s="3" t="n"/>
     </row>
     <row r="171">
-      <c r="A171" s="2" t="n"/>
+      <c r="A171" s="3" t="n"/>
     </row>
     <row r="172">
-      <c r="A172" s="2" t="n"/>
+      <c r="A172" s="3" t="n"/>
     </row>
     <row r="173">
-      <c r="A173" s="2" t="n"/>
+      <c r="A173" s="3" t="n"/>
     </row>
     <row r="174">
-      <c r="A174" s="2" t="n"/>
+      <c r="A174" s="3" t="n"/>
     </row>
     <row r="175">
-      <c r="A175" s="2" t="n"/>
+      <c r="A175" s="3" t="n"/>
     </row>
     <row r="176">
-      <c r="A176" s="2" t="n"/>
+      <c r="A176" s="3" t="n"/>
     </row>
     <row r="177">
-      <c r="A177" s="2" t="n"/>
+      <c r="A177" s="3" t="n"/>
     </row>
     <row r="178">
-      <c r="A178" s="2" t="n"/>
+      <c r="A178" s="3" t="n"/>
     </row>
     <row r="179">
-      <c r="A179" s="2" t="n"/>
+      <c r="A179" s="3" t="n"/>
     </row>
     <row r="180">
-      <c r="A180" s="2" t="n"/>
+      <c r="A180" s="3" t="n"/>
     </row>
     <row r="181">
-      <c r="A181" s="2" t="n"/>
+      <c r="A181" s="3" t="n"/>
     </row>
     <row r="182">
-      <c r="A182" s="2" t="n"/>
+      <c r="A182" s="3" t="n"/>
     </row>
     <row r="183">
-      <c r="A183" s="2" t="n"/>
+      <c r="A183" s="3" t="n"/>
     </row>
     <row r="184">
-      <c r="A184" s="2" t="n"/>
+      <c r="A184" s="3" t="n"/>
     </row>
     <row r="185">
-      <c r="A185" s="2" t="n"/>
+      <c r="A185" s="3" t="n"/>
     </row>
     <row r="186">
-      <c r="A186" s="2" t="n"/>
+      <c r="A186" s="3" t="n"/>
     </row>
     <row r="187">
-      <c r="A187" s="2" t="n"/>
+      <c r="A187" s="3" t="n"/>
     </row>
     <row r="188">
-      <c r="A188" s="2" t="n"/>
+      <c r="A188" s="3" t="n"/>
     </row>
     <row r="189">
-      <c r="A189" s="2" t="n"/>
+      <c r="A189" s="3" t="n"/>
     </row>
     <row r="190">
-      <c r="A190" s="2" t="n"/>
+      <c r="A190" s="3" t="n"/>
     </row>
     <row r="191">
-      <c r="A191" s="2" t="n"/>
+      <c r="A191" s="3" t="n"/>
     </row>
     <row r="192">
-      <c r="A192" s="2" t="n"/>
+      <c r="A192" s="3" t="n"/>
     </row>
     <row r="193">
-      <c r="A193" s="2" t="n"/>
+      <c r="A193" s="3" t="n"/>
     </row>
     <row r="194">
-      <c r="A194" s="2" t="n"/>
+      <c r="A194" s="3" t="n"/>
     </row>
     <row r="195">
-      <c r="A195" s="2" t="n"/>
+      <c r="A195" s="3" t="n"/>
     </row>
     <row r="196">
-      <c r="A196" s="2" t="n"/>
+      <c r="A196" s="3" t="n"/>
     </row>
     <row r="197">
-      <c r="A197" s="2" t="n"/>
+      <c r="A197" s="3" t="n"/>
     </row>
     <row r="198">
-      <c r="A198" s="2" t="n"/>
+      <c r="A198" s="3" t="n"/>
     </row>
     <row r="199">
-      <c r="A199" s="2" t="n"/>
+      <c r="A199" s="3" t="n"/>
     </row>
     <row r="200">
-      <c r="A200" s="2" t="n"/>
+      <c r="A200" s="3" t="n"/>
     </row>
     <row r="201">
-      <c r="A201" s="2" t="n"/>
+      <c r="A201" s="3" t="n"/>
     </row>
     <row r="202">
-      <c r="A202" s="2" t="n"/>
+      <c r="A202" s="3" t="n"/>
     </row>
     <row r="203">
-      <c r="A203" s="2" t="n"/>
+      <c r="A203" s="3" t="n"/>
     </row>
     <row r="204">
-      <c r="A204" s="2" t="n"/>
+      <c r="A204" s="3" t="n"/>
     </row>
     <row r="205">
-      <c r="A205" s="2" t="n"/>
+      <c r="A205" s="3" t="n"/>
     </row>
     <row r="206">
-      <c r="A206" s="2" t="n"/>
+      <c r="A206" s="3" t="n"/>
     </row>
     <row r="207">
-      <c r="A207" s="2" t="n"/>
+      <c r="A207" s="3" t="n"/>
     </row>
     <row r="208">
-      <c r="A208" s="2" t="n"/>
+      <c r="A208" s="3" t="n"/>
     </row>
     <row r="209">
-      <c r="A209" s="2" t="n"/>
+      <c r="A209" s="3" t="n"/>
     </row>
     <row r="210">
-      <c r="A210" s="2" t="n"/>
+      <c r="A210" s="3" t="n"/>
     </row>
     <row r="211">
-      <c r="A211" s="2" t="n"/>
+      <c r="A211" s="3" t="n"/>
     </row>
     <row r="212">
-      <c r="A212" s="2" t="n"/>
+      <c r="A212" s="3" t="n"/>
     </row>
     <row r="213">
-      <c r="A213" s="2" t="n"/>
+      <c r="A213" s="3" t="n"/>
     </row>
     <row r="214">
-      <c r="A214" s="2" t="n"/>
+      <c r="A214" s="3" t="n"/>
     </row>
     <row r="215">
-      <c r="A215" s="2" t="n"/>
+      <c r="A215" s="3" t="n"/>
     </row>
     <row r="216">
-      <c r="A216" s="2" t="n"/>
+      <c r="A216" s="3" t="n"/>
     </row>
     <row r="217">
-      <c r="A217" s="2" t="n"/>
+      <c r="A217" s="3" t="n"/>
     </row>
     <row r="218">
-      <c r="A218" s="2" t="n"/>
+      <c r="A218" s="3" t="n"/>
     </row>
     <row r="219">
-      <c r="A219" s="2" t="n"/>
+      <c r="A219" s="3" t="n"/>
     </row>
     <row r="220">
-      <c r="A220" s="2" t="n"/>
+      <c r="A220" s="3" t="n"/>
     </row>
     <row r="221">
-      <c r="A221" s="2" t="n"/>
+      <c r="A221" s="3" t="n"/>
     </row>
     <row r="222">
-      <c r="A222" s="2" t="n"/>
+      <c r="A222" s="3" t="n"/>
     </row>
     <row r="223">
-      <c r="A223" s="2" t="n"/>
+      <c r="A223" s="3" t="n"/>
     </row>
     <row r="224">
-      <c r="A224" s="2" t="n"/>
+      <c r="A224" s="3" t="n"/>
     </row>
     <row r="225">
-      <c r="A225" s="2" t="n"/>
+      <c r="A225" s="3" t="n"/>
     </row>
     <row r="226">
-      <c r="A226" s="2" t="n"/>
+      <c r="A226" s="3" t="n"/>
     </row>
     <row r="227">
-      <c r="A227" s="2" t="n"/>
+      <c r="A227" s="3" t="n"/>
     </row>
     <row r="228">
-      <c r="A228" s="2" t="n"/>
+      <c r="A228" s="3" t="n"/>
     </row>
     <row r="229">
-      <c r="A229" s="2" t="n"/>
+      <c r="A229" s="3" t="n"/>
     </row>
     <row r="230">
-      <c r="A230" s="2" t="n"/>
+      <c r="A230" s="3" t="n"/>
     </row>
     <row r="231">
-      <c r="A231" s="2" t="n"/>
+      <c r="A231" s="3" t="n"/>
     </row>
     <row r="232">
-      <c r="A232" s="2" t="n"/>
+      <c r="A232" s="3" t="n"/>
     </row>
     <row r="233">
-      <c r="A233" s="2" t="n"/>
+      <c r="A233" s="3" t="n"/>
     </row>
     <row r="234">
-      <c r="A234" s="2" t="n"/>
+      <c r="A234" s="3" t="n"/>
     </row>
     <row r="235">
-      <c r="A235" s="2" t="n"/>
+      <c r="A235" s="3" t="n"/>
     </row>
     <row r="236">
-      <c r="A236" s="2" t="n"/>
+      <c r="A236" s="3" t="n"/>
     </row>
     <row r="237">
-      <c r="A237" s="2" t="n"/>
+      <c r="A237" s="3" t="n"/>
     </row>
     <row r="238">
-      <c r="A238" s="2" t="n"/>
+      <c r="A238" s="3" t="n"/>
     </row>
     <row r="239">
-      <c r="A239" s="2" t="n"/>
+      <c r="A239" s="3" t="n"/>
     </row>
     <row r="240">
-      <c r="A240" s="2" t="n"/>
+      <c r="A240" s="3" t="n"/>
     </row>
     <row r="241">
-      <c r="A241" s="2" t="n"/>
+      <c r="A241" s="3" t="n"/>
     </row>
     <row r="242">
-      <c r="A242" s="2" t="n"/>
+      <c r="A242" s="3" t="n"/>
     </row>
     <row r="243">
-      <c r="A243" s="2" t="n"/>
+      <c r="A243" s="3" t="n"/>
     </row>
     <row r="244">
-      <c r="A244" s="2" t="n"/>
+      <c r="A244" s="3" t="n"/>
     </row>
     <row r="245">
-      <c r="A245" s="2" t="n"/>
+      <c r="A245" s="3" t="n"/>
     </row>
     <row r="246">
-      <c r="A246" s="2" t="n"/>
+      <c r="A246" s="3" t="n"/>
     </row>
     <row r="247">
-      <c r="A247" s="2" t="n"/>
+      <c r="A247" s="3" t="n"/>
     </row>
     <row r="248">
-      <c r="A248" s="2" t="n"/>
+      <c r="A248" s="3" t="n"/>
     </row>
     <row r="249">
-      <c r="A249" s="2" t="n"/>
+      <c r="A249" s="3" t="n"/>
     </row>
     <row r="250">
-      <c r="A250" s="2" t="n"/>
+      <c r="A250" s="3" t="n"/>
     </row>
     <row r="251">
-      <c r="A251" s="2" t="n"/>
+      <c r="A251" s="3" t="n"/>
     </row>
     <row r="252">
-      <c r="A252" s="2" t="n"/>
+      <c r="A252" s="3" t="n"/>
     </row>
     <row r="253">
-      <c r="A253" s="2" t="n"/>
+      <c r="A253" s="3" t="n"/>
     </row>
     <row r="254">
-      <c r="A254" s="2" t="n"/>
+      <c r="A254" s="3" t="n"/>
     </row>
     <row r="255">
-      <c r="A255" s="2" t="n"/>
+      <c r="A255" s="3" t="n"/>
     </row>
     <row r="256">
-      <c r="A256" s="2" t="n"/>
+      <c r="A256" s="3" t="n"/>
     </row>
     <row r="257">
-      <c r="A257" s="2" t="n"/>
+      <c r="A257" s="3" t="n"/>
     </row>
     <row r="258">
-      <c r="A258" s="2" t="n"/>
+      <c r="A258" s="3" t="n"/>
     </row>
     <row r="259">
-      <c r="A259" s="2" t="n"/>
+      <c r="A259" s="3" t="n"/>
     </row>
     <row r="260">
-      <c r="A260" s="2" t="n"/>
+      <c r="A260" s="3" t="n"/>
     </row>
     <row r="261">
-      <c r="A261" s="2" t="n"/>
+      <c r="A261" s="3" t="n"/>
     </row>
     <row r="262">
-      <c r="A262" s="2" t="n"/>
+      <c r="A262" s="3" t="n"/>
     </row>
     <row r="263">
-      <c r="A263" s="2" t="n"/>
+      <c r="A263" s="3" t="n"/>
     </row>
     <row r="264">
-      <c r="A264" s="2" t="n"/>
+      <c r="A264" s="3" t="n"/>
     </row>
     <row r="265">
-      <c r="A265" s="2" t="n"/>
+      <c r="A265" s="3" t="n"/>
     </row>
     <row r="266">
-      <c r="A266" s="2" t="n"/>
+      <c r="A266" s="3" t="n"/>
     </row>
     <row r="267">
-      <c r="A267" s="2" t="n"/>
+      <c r="A267" s="3" t="n"/>
     </row>
     <row r="268">
-      <c r="A268" s="2" t="n"/>
+      <c r="A268" s="3" t="n"/>
     </row>
     <row r="269">
-      <c r="A269" s="2" t="n"/>
+      <c r="A269" s="3" t="n"/>
     </row>
     <row r="270">
-      <c r="A270" s="2" t="n"/>
+      <c r="A270" s="3" t="n"/>
     </row>
     <row r="271">
-      <c r="A271" s="2" t="n"/>
+      <c r="A271" s="3" t="n"/>
     </row>
     <row r="272">
-      <c r="A272" s="2" t="n"/>
+      <c r="A272" s="3" t="n"/>
     </row>
     <row r="273">
-      <c r="A273" s="2" t="n"/>
+      <c r="A273" s="3" t="n"/>
     </row>
     <row r="274">
-      <c r="A274" s="2" t="n"/>
+      <c r="A274" s="3" t="n"/>
     </row>
     <row r="275">
-      <c r="A275" s="2" t="n"/>
+      <c r="A275" s="3" t="n"/>
     </row>
     <row r="276">
-      <c r="A276" s="2" t="n"/>
+      <c r="A276" s="3" t="n"/>
     </row>
     <row r="277">
-      <c r="A277" s="2" t="n"/>
+      <c r="A277" s="3" t="n"/>
     </row>
     <row r="278">
-      <c r="A278" s="2" t="n"/>
+      <c r="A278" s="3" t="n"/>
     </row>
     <row r="279">
-      <c r="A279" s="2" t="n"/>
+      <c r="A279" s="3" t="n"/>
     </row>
     <row r="280">
-      <c r="A280" s="2" t="n"/>
+      <c r="A280" s="3" t="n"/>
     </row>
     <row r="281">
-      <c r="A281" s="2" t="n"/>
+      <c r="A281" s="3" t="n"/>
     </row>
     <row r="282">
-      <c r="A282" s="2" t="n"/>
+      <c r="A282" s="3" t="n"/>
     </row>
     <row r="283">
-      <c r="A283" s="2" t="n"/>
+      <c r="A283" s="3" t="n"/>
     </row>
     <row r="284">
-      <c r="A284" s="2" t="n"/>
+      <c r="A284" s="3" t="n"/>
     </row>
     <row r="285">
-      <c r="A285" s="2" t="n"/>
+      <c r="A285" s="3" t="n"/>
     </row>
     <row r="286">
-      <c r="A286" s="2" t="n"/>
+      <c r="A286" s="3" t="n"/>
     </row>
     <row r="287">
-      <c r="A287" s="2" t="n"/>
+      <c r="A287" s="3" t="n"/>
     </row>
     <row r="288">
-      <c r="A288" s="2" t="n"/>
+      <c r="A288" s="3" t="n"/>
     </row>
     <row r="289">
-      <c r="A289" s="2" t="n"/>
+      <c r="A289" s="3" t="n"/>
     </row>
     <row r="290">
-      <c r="A290" s="2" t="n"/>
+      <c r="A290" s="3" t="n"/>
     </row>
     <row r="291">
-      <c r="A291" s="2" t="n"/>
+      <c r="A291" s="3" t="n"/>
     </row>
     <row r="292">
-      <c r="A292" s="2" t="n"/>
+      <c r="A292" s="3" t="n"/>
     </row>
     <row r="293">
-      <c r="A293" s="2" t="n"/>
+      <c r="A293" s="3" t="n"/>
     </row>
     <row r="294">
-      <c r="A294" s="2" t="n"/>
+      <c r="A294" s="3" t="n"/>
     </row>
     <row r="295">
-      <c r="A295" s="2" t="n"/>
+      <c r="A295" s="3" t="n"/>
     </row>
     <row r="296">
-      <c r="A296" s="2" t="n"/>
+      <c r="A296" s="3" t="n"/>
     </row>
     <row r="297">
-      <c r="A297" s="2" t="n"/>
+      <c r="A297" s="3" t="n"/>
     </row>
     <row r="298">
-      <c r="A298" s="2" t="n"/>
+      <c r="A298" s="3" t="n"/>
     </row>
     <row r="299">
-      <c r="A299" s="2" t="n"/>
+      <c r="A299" s="3" t="n"/>
     </row>
     <row r="300">
-      <c r="A300" s="2" t="n"/>
+      <c r="A300" s="3" t="n"/>
     </row>
     <row r="301">
-      <c r="A301" s="2" t="n"/>
+      <c r="A301" s="3" t="n"/>
     </row>
     <row r="302">
-      <c r="A302" s="2" t="n"/>
+      <c r="A302" s="3" t="n"/>
     </row>
     <row r="303">
-      <c r="A303" s="2" t="n"/>
+      <c r="A303" s="3" t="n"/>
     </row>
     <row r="304">
-      <c r="A304" s="2" t="n"/>
+      <c r="A304" s="3" t="n"/>
     </row>
     <row r="305">
-      <c r="A305" s="2" t="n"/>
+      <c r="A305" s="3" t="n"/>
     </row>
     <row r="306">
-      <c r="A306" s="2" t="n"/>
+      <c r="A306" s="3" t="n"/>
     </row>
     <row r="307">
-      <c r="A307" s="2" t="n"/>
+      <c r="A307" s="3" t="n"/>
     </row>
     <row r="308">
-      <c r="A308" s="2" t="n"/>
+      <c r="A308" s="3" t="n"/>
     </row>
     <row r="309">
-      <c r="A309" s="2" t="n"/>
+      <c r="A309" s="3" t="n"/>
     </row>
     <row r="310">
-      <c r="A310" s="2" t="n"/>
+      <c r="A310" s="3" t="n"/>
     </row>
     <row r="311">
-      <c r="A311" s="2" t="n"/>
+      <c r="A311" s="3" t="n"/>
     </row>
     <row r="312">
-      <c r="A312" s="2" t="n"/>
+      <c r="A312" s="3" t="n"/>
     </row>
     <row r="313">
-      <c r="A313" s="2" t="n"/>
+      <c r="A313" s="3" t="n"/>
     </row>
     <row r="314">
-      <c r="A314" s="2" t="n"/>
+      <c r="A314" s="3" t="n"/>
     </row>
     <row r="315">
-      <c r="A315" s="2" t="n"/>
+      <c r="A315" s="3" t="n"/>
     </row>
     <row r="316">
-      <c r="A316" s="2" t="n"/>
+      <c r="A316" s="3" t="n"/>
     </row>
     <row r="317">
-      <c r="A317" s="2" t="n"/>
+      <c r="A317" s="3" t="n"/>
     </row>
     <row r="318">
-      <c r="A318" s="2" t="n"/>
+      <c r="A318" s="3" t="n"/>
     </row>
     <row r="319">
-      <c r="A319" s="2" t="n"/>
+      <c r="A319" s="3" t="n"/>
     </row>
     <row r="320">
-      <c r="A320" s="2" t="n"/>
+      <c r="A320" s="3" t="n"/>
     </row>
     <row r="321">
-      <c r="A321" s="2" t="n"/>
+      <c r="A321" s="3" t="n"/>
     </row>
     <row r="322">
-      <c r="A322" s="2" t="n"/>
+      <c r="A322" s="3" t="n"/>
     </row>
     <row r="323">
-      <c r="A323" s="2" t="n"/>
+      <c r="A323" s="3" t="n"/>
     </row>
     <row r="324">
-      <c r="A324" s="2" t="n"/>
+      <c r="A324" s="3" t="n"/>
     </row>
     <row r="325">
-      <c r="A325" s="2" t="n"/>
+      <c r="A325" s="3" t="n"/>
     </row>
     <row r="326">
-      <c r="A326" s="2" t="n"/>
+      <c r="A326" s="3" t="n"/>
     </row>
     <row r="327">
-      <c r="A327" s="2" t="n"/>
+      <c r="A327" s="3" t="n"/>
     </row>
     <row r="328">
-      <c r="A328" s="2" t="n"/>
+      <c r="A328" s="3" t="n"/>
     </row>
     <row r="329">
-      <c r="A329" s="2" t="n"/>
+      <c r="A329" s="3" t="n"/>
     </row>
     <row r="330">
-      <c r="A330" s="2" t="n"/>
+      <c r="A330" s="3" t="n"/>
     </row>
     <row r="331">
-      <c r="A331" s="2" t="n"/>
+      <c r="A331" s="3" t="n"/>
     </row>
     <row r="332">
-      <c r="A332" s="2" t="n"/>
+      <c r="A332" s="3" t="n"/>
     </row>
     <row r="333">
-      <c r="A333" s="2" t="n"/>
+      <c r="A333" s="3" t="n"/>
     </row>
     <row r="334">
-      <c r="A334" s="2" t="n"/>
+      <c r="A334" s="3" t="n"/>
     </row>
     <row r="335">
-      <c r="A335" s="2" t="n"/>
+      <c r="A335" s="3" t="n"/>
     </row>
     <row r="336">
-      <c r="A336" s="2" t="n"/>
+      <c r="A336" s="3" t="n"/>
     </row>
     <row r="337">
-      <c r="A337" s="2" t="n"/>
+      <c r="A337" s="3" t="n"/>
     </row>
     <row r="338">
-      <c r="A338" s="2" t="n"/>
+      <c r="A338" s="3" t="n"/>
     </row>
     <row r="339">
-      <c r="A339" s="2" t="n"/>
+      <c r="A339" s="3" t="n"/>
     </row>
     <row r="340">
-      <c r="A340" s="2" t="n"/>
+      <c r="A340" s="3" t="n"/>
     </row>
     <row r="341">
-      <c r="A341" s="2" t="n"/>
+      <c r="A341" s="3" t="n"/>
     </row>
     <row r="342">
-      <c r="A342" s="2" t="n"/>
+      <c r="A342" s="3" t="n"/>
     </row>
     <row r="343">
-      <c r="A343" s="2" t="n"/>
+      <c r="A343" s="3" t="n"/>
     </row>
     <row r="344">
-      <c r="A344" s="2" t="n"/>
+      <c r="A344" s="3" t="n"/>
     </row>
     <row r="345">
-      <c r="A345" s="2" t="n"/>
+      <c r="A345" s="3" t="n"/>
     </row>
     <row r="346">
-      <c r="A346" s="2" t="n"/>
+      <c r="A346" s="3" t="n"/>
     </row>
     <row r="347">
-      <c r="A347" s="2" t="n"/>
+      <c r="A347" s="3" t="n"/>
     </row>
     <row r="348">
-      <c r="A348" s="2" t="n"/>
+      <c r="A348" s="3" t="n"/>
     </row>
     <row r="349">
-      <c r="A349" s="2" t="n"/>
+      <c r="A349" s="3" t="n"/>
     </row>
     <row r="350">
-      <c r="A350" s="2" t="n"/>
+      <c r="A350" s="3" t="n"/>
     </row>
     <row r="351">
-      <c r="A351" s="2" t="n"/>
+      <c r="A351" s="3" t="n"/>
     </row>
     <row r="352">
-      <c r="A352" s="2" t="n"/>
+      <c r="A352" s="3" t="n"/>
     </row>
     <row r="353">
-      <c r="A353" s="2" t="n"/>
+      <c r="A353" s="3" t="n"/>
     </row>
     <row r="354">
-      <c r="A354" s="2" t="n"/>
+      <c r="A354" s="3" t="n"/>
     </row>
     <row r="355">
-      <c r="A355" s="2" t="n"/>
+      <c r="A355" s="3" t="n"/>
     </row>
     <row r="356">
-      <c r="A356" s="2" t="n"/>
+      <c r="A356" s="3" t="n"/>
     </row>
     <row r="357">
-      <c r="A357" s="2" t="n"/>
+      <c r="A357" s="3" t="n"/>
     </row>
     <row r="358">
-      <c r="A358" s="2" t="n"/>
+      <c r="A358" s="3" t="n"/>
     </row>
     <row r="359">
-      <c r="A359" s="2" t="n"/>
+      <c r="A359" s="3" t="n"/>
     </row>
     <row r="360">
-      <c r="A360" s="2" t="n"/>
+      <c r="A360" s="3" t="n"/>
     </row>
     <row r="361">
-      <c r="A361" s="2" t="n"/>
+      <c r="A361" s="3" t="n"/>
     </row>
     <row r="362">
-      <c r="A362" s="2" t="n"/>
+      <c r="A362" s="3" t="n"/>
     </row>
     <row r="363">
-      <c r="A363" s="2" t="n"/>
+      <c r="A363" s="3" t="n"/>
     </row>
     <row r="364">
-      <c r="A364" s="2" t="n"/>
+      <c r="A364" s="3" t="n"/>
     </row>
     <row r="365">
-      <c r="A365" s="2" t="n"/>
+      <c r="A365" s="3" t="n"/>
     </row>
     <row r="366">
-      <c r="A366" s="2" t="n"/>
+      <c r="A366" s="3" t="n"/>
     </row>
     <row r="367">
-      <c r="A367" s="2" t="n"/>
+      <c r="A367" s="3" t="n"/>
     </row>
     <row r="368">
-      <c r="A368" s="2" t="n"/>
+      <c r="A368" s="3" t="n"/>
     </row>
     <row r="369">
-      <c r="A369" s="2" t="n"/>
+      <c r="A369" s="3" t="n"/>
     </row>
     <row r="370">
-      <c r="A370" s="2" t="n"/>
+      <c r="A370" s="3" t="n"/>
     </row>
     <row r="371">
-      <c r="A371" s="2" t="n"/>
+      <c r="A371" s="3" t="n"/>
     </row>
     <row r="372">
-      <c r="A372" s="2" t="n"/>
+      <c r="A372" s="3" t="n"/>
     </row>
     <row r="373">
-      <c r="A373" s="2" t="n"/>
+      <c r="A373" s="3" t="n"/>
     </row>
     <row r="374">
-      <c r="A374" s="2" t="n"/>
+      <c r="A374" s="3" t="n"/>
     </row>
     <row r="375">
-      <c r="A375" s="2" t="n"/>
+      <c r="A375" s="3" t="n"/>
     </row>
     <row r="376">
-      <c r="A376" s="2" t="n"/>
+      <c r="A376" s="3" t="n"/>
     </row>
     <row r="377">
-      <c r="A377" s="2" t="n"/>
+      <c r="A377" s="3" t="n"/>
     </row>
     <row r="378">
-      <c r="A378" s="2" t="n"/>
+      <c r="A378" s="3" t="n"/>
     </row>
     <row r="379">
-      <c r="A379" s="2" t="n"/>
+      <c r="A379" s="3" t="n"/>
     </row>
     <row r="380">
-      <c r="A380" s="2" t="n"/>
+      <c r="A380" s="3" t="n"/>
     </row>
     <row r="381">
-      <c r="A381" s="2" t="n"/>
+      <c r="A381" s="3" t="n"/>
     </row>
     <row r="382">
-      <c r="A382" s="2" t="n"/>
+      <c r="A382" s="3" t="n"/>
     </row>
     <row r="383">
-      <c r="A383" s="2" t="n"/>
+      <c r="A383" s="3" t="n"/>
     </row>
     <row r="384">
-      <c r="A384" s="2" t="n"/>
+      <c r="A384" s="3" t="n"/>
     </row>
     <row r="385">
-      <c r="A385" s="2" t="n"/>
+      <c r="A385" s="3" t="n"/>
     </row>
     <row r="386">
-      <c r="A386" s="2" t="n"/>
+      <c r="A386" s="3" t="n"/>
     </row>
     <row r="387">
-      <c r="A387" s="2" t="n"/>
+      <c r="A387" s="3" t="n"/>
     </row>
     <row r="388">
-      <c r="A388" s="2" t="n"/>
+      <c r="A388" s="3" t="n"/>
     </row>
     <row r="389">
-      <c r="A389" s="2" t="n"/>
+      <c r="A389" s="3" t="n"/>
     </row>
     <row r="390">
-      <c r="A390" s="2" t="n"/>
+      <c r="A390" s="3" t="n"/>
     </row>
     <row r="391">
-      <c r="A391" s="2" t="n"/>
+      <c r="A391" s="3" t="n"/>
     </row>
     <row r="392">
-      <c r="A392" s="2" t="n"/>
+      <c r="A392" s="3" t="n"/>
     </row>
     <row r="393">
-      <c r="A393" s="2" t="n"/>
+      <c r="A393" s="3" t="n"/>
     </row>
     <row r="394">
-      <c r="A394" s="2" t="n"/>
+      <c r="A394" s="3" t="n"/>
     </row>
     <row r="395">
-      <c r="A395" s="2" t="n"/>
+      <c r="A395" s="3" t="n"/>
     </row>
     <row r="396">
-      <c r="A396" s="2" t="n"/>
+      <c r="A396" s="3" t="n"/>
     </row>
     <row r="397">
-      <c r="A397" s="2" t="n"/>
+      <c r="A397" s="3" t="n"/>
     </row>
     <row r="398">
-      <c r="A398" s="2" t="n"/>
+      <c r="A398" s="3" t="n"/>
     </row>
     <row r="399">
-      <c r="A399" s="2" t="n"/>
+      <c r="A399" s="3" t="n"/>
     </row>
     <row r="400">
-      <c r="A400" s="2" t="n"/>
+      <c r="A400" s="3" t="n"/>
     </row>
     <row r="401">
-      <c r="A401" s="2" t="n"/>
+      <c r="A401" s="3" t="n"/>
     </row>
     <row r="402">
-      <c r="A402" s="2" t="n"/>
+      <c r="A402" s="3" t="n"/>
     </row>
     <row r="403">
-      <c r="A403" s="2" t="n"/>
+      <c r="A403" s="3" t="n"/>
     </row>
     <row r="404">
-      <c r="A404" s="2" t="n"/>
+      <c r="A404" s="3" t="n"/>
     </row>
     <row r="405">
-      <c r="A405" s="2" t="n"/>
+      <c r="A405" s="3" t="n"/>
     </row>
     <row r="406">
-      <c r="A406" s="2" t="n"/>
+      <c r="A406" s="3" t="n"/>
     </row>
     <row r="407">
-      <c r="A407" s="2" t="n"/>
+      <c r="A407" s="3" t="n"/>
     </row>
     <row r="408">
-      <c r="A408" s="2" t="n"/>
+      <c r="A408" s="3" t="n"/>
     </row>
     <row r="409">
-      <c r="A409" s="2" t="n"/>
+      <c r="A409" s="3" t="n"/>
     </row>
     <row r="410">
-      <c r="A410" s="2" t="n"/>
+      <c r="A410" s="3" t="n"/>
     </row>
     <row r="411">
-      <c r="A411" s="2" t="n"/>
+      <c r="A411" s="3" t="n"/>
     </row>
     <row r="412">
-      <c r="A412" s="2" t="n"/>
+      <c r="A412" s="3" t="n"/>
     </row>
     <row r="413">
-      <c r="A413" s="2" t="n"/>
+      <c r="A413" s="3" t="n"/>
     </row>
     <row r="414">
-      <c r="A414" s="2" t="n"/>
+      <c r="A414" s="3" t="n"/>
     </row>
     <row r="415">
-      <c r="A415" s="2" t="n"/>
+      <c r="A415" s="3" t="n"/>
     </row>
     <row r="416">
-      <c r="A416" s="2" t="n"/>
+      <c r="A416" s="3" t="n"/>
     </row>
     <row r="417">
-      <c r="A417" s="2" t="n"/>
+      <c r="A417" s="3" t="n"/>
     </row>
     <row r="418">
-      <c r="A418" s="2" t="n"/>
+      <c r="A418" s="3" t="n"/>
     </row>
     <row r="419">
-      <c r="A419" s="2" t="n"/>
+      <c r="A419" s="3" t="n"/>
     </row>
     <row r="420">
-      <c r="A420" s="2" t="n"/>
+      <c r="A420" s="3" t="n"/>
     </row>
     <row r="421">
-      <c r="A421" s="2" t="n"/>
+      <c r="A421" s="3" t="n"/>
     </row>
     <row r="422">
-      <c r="A422" s="2" t="n"/>
+      <c r="A422" s="3" t="n"/>
     </row>
     <row r="423">
-      <c r="A423" s="2" t="n"/>
+      <c r="A423" s="3" t="n"/>
     </row>
     <row r="424">
-      <c r="A424" s="2" t="n"/>
+      <c r="A424" s="3" t="n"/>
     </row>
     <row r="425">
-      <c r="A425" s="2" t="n"/>
+      <c r="A425" s="3" t="n"/>
     </row>
     <row r="426">
-      <c r="A426" s="2" t="n"/>
+      <c r="A426" s="3" t="n"/>
     </row>
     <row r="427">
-      <c r="A427" s="2" t="n"/>
+      <c r="A427" s="3" t="n"/>
     </row>
     <row r="428">
-      <c r="A428" s="2" t="n"/>
+      <c r="A428" s="3" t="n"/>
     </row>
     <row r="429">
-      <c r="A429" s="2" t="n"/>
+      <c r="A429" s="3" t="n"/>
     </row>
     <row r="430">
-      <c r="A430" s="2" t="n"/>
+      <c r="A430" s="3" t="n"/>
     </row>
     <row r="431">
-      <c r="A431" s="2" t="n"/>
+      <c r="A431" s="3" t="n"/>
     </row>
     <row r="432">
-      <c r="A432" s="2" t="n"/>
+      <c r="A432" s="3" t="n"/>
     </row>
     <row r="433">
-      <c r="A433" s="2" t="n"/>
+      <c r="A433" s="3" t="n"/>
     </row>
     <row r="434">
-      <c r="A434" s="2" t="n"/>
+      <c r="A434" s="3" t="n"/>
     </row>
     <row r="435">
-      <c r="A435" s="2" t="n"/>
+      <c r="A435" s="3" t="n"/>
     </row>
     <row r="436">
-      <c r="A436" s="2" t="n"/>
+      <c r="A436" s="3" t="n"/>
     </row>
     <row r="437">
-      <c r="A437" s="2" t="n"/>
+      <c r="A437" s="3" t="n"/>
     </row>
     <row r="438">
-      <c r="A438" s="2" t="n"/>
+      <c r="A438" s="3" t="n"/>
     </row>
     <row r="439">
-      <c r="A439" s="2" t="n"/>
+      <c r="A439" s="3" t="n"/>
     </row>
     <row r="440">
-      <c r="A440" s="2" t="n"/>
+      <c r="A440" s="3" t="n"/>
     </row>
     <row r="441">
-      <c r="A441" s="2" t="n"/>
+      <c r="A441" s="3" t="n"/>
     </row>
     <row r="442">
-      <c r="A442" s="2" t="n"/>
+      <c r="A442" s="3" t="n"/>
     </row>
     <row r="443">
-      <c r="A443" s="2" t="n"/>
+      <c r="A443" s="3" t="n"/>
     </row>
     <row r="444">
-      <c r="A444" s="2" t="n"/>
+      <c r="A444" s="3" t="n"/>
     </row>
     <row r="445">
-      <c r="A445" s="2" t="n"/>
+      <c r="A445" s="3" t="n"/>
     </row>
     <row r="446">
-      <c r="A446" s="2" t="n"/>
+      <c r="A446" s="3" t="n"/>
     </row>
     <row r="447">
-      <c r="A447" s="2" t="n"/>
+      <c r="A447" s="3" t="n"/>
     </row>
     <row r="448">
-      <c r="A448" s="2" t="n"/>
+      <c r="A448" s="3" t="n"/>
     </row>
     <row r="449">
-      <c r="A449" s="2" t="n"/>
+      <c r="A449" s="3" t="n"/>
     </row>
     <row r="450">
-      <c r="A450" s="2" t="n"/>
+      <c r="A450" s="3" t="n"/>
     </row>
     <row r="451">
-      <c r="A451" s="2" t="n"/>
+      <c r="A451" s="3" t="n"/>
     </row>
     <row r="452">
-      <c r="A452" s="2" t="n"/>
+      <c r="A452" s="3" t="n"/>
     </row>
     <row r="453">
-      <c r="A453" s="2" t="n"/>
+      <c r="A453" s="3" t="n"/>
     </row>
     <row r="454">
-      <c r="A454" s="2" t="n"/>
+      <c r="A454" s="3" t="n"/>
     </row>
     <row r="455">
-      <c r="A455" s="2" t="n"/>
+      <c r="A455" s="3" t="n"/>
     </row>
     <row r="456">
-      <c r="A456" s="2" t="n"/>
+      <c r="A456" s="3" t="n"/>
     </row>
     <row r="457">
-      <c r="A457" s="2" t="n"/>
+      <c r="A457" s="3" t="n"/>
     </row>
     <row r="458">
-      <c r="A458" s="2" t="n"/>
+      <c r="A458" s="3" t="n"/>
     </row>
     <row r="459">
-      <c r="A459" s="2" t="n"/>
+      <c r="A459" s="3" t="n"/>
     </row>
     <row r="460">
-      <c r="A460" s="2" t="n"/>
+      <c r="A460" s="3" t="n"/>
     </row>
     <row r="461">
-      <c r="A461" s="2" t="n"/>
+      <c r="A461" s="3" t="n"/>
     </row>
     <row r="462">
-      <c r="A462" s="2" t="n"/>
+      <c r="A462" s="3" t="n"/>
     </row>
     <row r="463">
-      <c r="A463" s="2" t="n"/>
+      <c r="A463" s="3" t="n"/>
     </row>
     <row r="464">
-      <c r="A464" s="2" t="n"/>
+      <c r="A464" s="3" t="n"/>
     </row>
     <row r="465">
-      <c r="A465" s="2" t="n"/>
+      <c r="A465" s="3" t="n"/>
     </row>
     <row r="466">
-      <c r="A466" s="2" t="n"/>
+      <c r="A466" s="3" t="n"/>
     </row>
     <row r="467">
-      <c r="A467" s="2" t="n"/>
+      <c r="A467" s="3" t="n"/>
     </row>
     <row r="468">
-      <c r="A468" s="2" t="n"/>
+      <c r="A468" s="3" t="n"/>
     </row>
     <row r="469">
-      <c r="A469" s="2" t="n"/>
+      <c r="A469" s="3" t="n"/>
     </row>
     <row r="470">
-      <c r="A470" s="2" t="n"/>
+      <c r="A470" s="3" t="n"/>
     </row>
     <row r="471">
-      <c r="A471" s="2" t="n"/>
+      <c r="A471" s="3" t="n"/>
     </row>
     <row r="472">
-      <c r="A472" s="2" t="n"/>
+      <c r="A472" s="3" t="n"/>
     </row>
     <row r="473">
-      <c r="A473" s="2" t="n"/>
+      <c r="A473" s="3" t="n"/>
     </row>
     <row r="474">
-      <c r="A474" s="2" t="n"/>
+      <c r="A474" s="3" t="n"/>
     </row>
     <row r="475">
-      <c r="A475" s="2" t="n"/>
+      <c r="A475" s="3" t="n"/>
     </row>
     <row r="476">
-      <c r="A476" s="2" t="n"/>
+      <c r="A476" s="3" t="n"/>
     </row>
     <row r="477">
-      <c r="A477" s="2" t="n"/>
+      <c r="A477" s="3" t="n"/>
     </row>
     <row r="478">
-      <c r="A478" s="2" t="n"/>
+      <c r="A478" s="3" t="n"/>
     </row>
     <row r="479">
-      <c r="A479" s="2" t="n"/>
+      <c r="A479" s="3" t="n"/>
     </row>
     <row r="480">
-      <c r="A480" s="2" t="n"/>
+      <c r="A480" s="3" t="n"/>
     </row>
     <row r="481">
-      <c r="A481" s="2" t="n"/>
+      <c r="A481" s="3" t="n"/>
     </row>
     <row r="482">
-      <c r="A482" s="2" t="n"/>
+      <c r="A482" s="3" t="n"/>
     </row>
     <row r="483">
-      <c r="A483" s="2" t="n"/>
+      <c r="A483" s="3" t="n"/>
     </row>
     <row r="484">
-      <c r="A484" s="2" t="n"/>
+      <c r="A484" s="3" t="n"/>
     </row>
     <row r="485">
-      <c r="A485" s="2" t="n"/>
+      <c r="A485" s="3" t="n"/>
     </row>
     <row r="486">
-      <c r="A486" s="2" t="n"/>
+      <c r="A486" s="3" t="n"/>
     </row>
     <row r="487">
-      <c r="A487" s="2" t="n"/>
+      <c r="A487" s="3" t="n"/>
     </row>
     <row r="488">
-      <c r="A488" s="2" t="n"/>
+      <c r="A488" s="3" t="n"/>
     </row>
     <row r="489">
-      <c r="A489" s="2" t="n"/>
+      <c r="A489" s="3" t="n"/>
     </row>
     <row r="490">
-      <c r="A490" s="2" t="n"/>
+      <c r="A490" s="3" t="n"/>
     </row>
     <row r="491">
-      <c r="A491" s="2" t="n"/>
+      <c r="A491" s="3" t="n"/>
     </row>
     <row r="492">
-      <c r="A492" s="2" t="n"/>
+      <c r="A492" s="3" t="n"/>
     </row>
     <row r="493">
-      <c r="A493" s="2" t="n"/>
+      <c r="A493" s="3" t="n"/>
     </row>
     <row r="494">
-      <c r="A494" s="2" t="n"/>
+      <c r="A494" s="3" t="n"/>
     </row>
     <row r="495">
-      <c r="A495" s="2" t="n"/>
+      <c r="A495" s="3" t="n"/>
     </row>
     <row r="496">
-      <c r="A496" s="2" t="n"/>
+      <c r="A496" s="3" t="n"/>
     </row>
     <row r="497">
-      <c r="A497" s="2" t="n"/>
+      <c r="A497" s="3" t="n"/>
     </row>
     <row r="498">
-      <c r="A498" s="2" t="n"/>
+      <c r="A498" s="3" t="n"/>
     </row>
     <row r="499">
-      <c r="A499" s="2" t="n"/>
+      <c r="A499" s="3" t="n"/>
     </row>
     <row r="500">
-      <c r="A500" s="2" t="n"/>
+      <c r="A500" s="3" t="n"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -2014,26 +2109,26 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C16"/>
+  <dimension ref="A1:C20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="14" customWidth="1" min="1" max="1"/>
-    <col width="66" customWidth="1" min="2" max="2"/>
+    <col width="18" customWidth="1" min="1" max="1"/>
+    <col width="70" customWidth="1" min="2" max="2"/>
     <col width="24" customWidth="1" min="3" max="3"/>
   </cols>
   <sheetData>
     <row r="1">
-      <c r="A1" s="3" t="inlineStr">
+      <c r="A1" s="4" t="inlineStr">
         <is>
           <t>Column</t>
         </is>
       </c>
-      <c r="B1" s="3" t="inlineStr">
+      <c r="B1" s="4" t="inlineStr">
         <is>
           <t>What to type</t>
         </is>
       </c>
-      <c r="C1" s="3" t="inlineStr">
+      <c r="C1" s="4" t="inlineStr">
         <is>
           <t>Example</t>
         </is>
@@ -2227,40 +2322,100 @@
       </c>
     </row>
     <row r="13">
-      <c r="A13" t="inlineStr"/>
-      <c r="B13" t="inlineStr"/>
-      <c r="C13" t="inlineStr"/>
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>Safety Bar Squat</t>
+        </is>
+      </c>
+      <c r="B13" t="inlineStr">
+        <is>
+          <t>Weight x reps, 1-10 reps.</t>
+        </is>
+      </c>
+      <c r="C13" t="inlineStr">
+        <is>
+          <t>335x5</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>Tips</t>
+          <t>Push-Up</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>Leave a cell blank if the athlete did not test.</t>
-        </is>
-      </c>
-      <c r="C14" t="inlineStr"/>
+          <t>Number of reps.</t>
+        </is>
+      </c>
+      <c r="C14" t="inlineStr">
+        <is>
+          <t>31</t>
+        </is>
+      </c>
     </row>
     <row r="15">
-      <c r="A15" t="inlineStr"/>
+      <c r="A15" t="inlineStr">
+        <is>
+          <t>Chin-Up</t>
+        </is>
+      </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>Delete any test column your team does not use.</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr"/>
+          <t>Number of reps.</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>7</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr"/>
-      <c r="B16" t="inlineStr">
+      <c r="B16" t="inlineStr"/>
+      <c r="C16" t="inlineStr"/>
+    </row>
+    <row r="17">
+      <c r="A17" t="inlineStr">
+        <is>
+          <t>Tips</t>
+        </is>
+      </c>
+      <c r="B17" t="inlineStr">
+        <is>
+          <t>Row 2 (gray) shows how to type each column. Leave it. The website skips it.</t>
+        </is>
+      </c>
+      <c r="C17" t="inlineStr"/>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr"/>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>Leave a cell blank if the athlete did not test.</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr"/>
+      <c r="B19" t="inlineStr">
+        <is>
+          <t>Delete any test column your team does not use.</t>
+        </is>
+      </c>
+      <c r="C19" t="inlineStr"/>
+    </row>
+    <row r="20">
+      <c r="A20" t="inlineStr"/>
+      <c r="B20" t="inlineStr">
         <is>
           <t>Keep the header names as they are. Column order does not matter.</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr"/>
+      <c r="C20" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>